<commit_message>
Tokens y Actualizaciones de las hojas
</commit_message>
<xml_diff>
--- a/Sheets/One-Shot Premades/Arcanista.xlsx
+++ b/Sheets/One-Shot Premades/Arcanista.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="A:\Javier\TTRPGs\Marvel Multiverse\Sheets\One-Shot Premades\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="A:\Javier\TTRPGs\Marvel Multiverse RPG\Sheets\One-Shot Premades\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{194B4213-5A1E-414B-AA68-F1E51D76C990}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{749A85E7-AC16-4E87-BA6F-45BA7F3B38C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Frente" sheetId="1" r:id="rId1"/>
@@ -291,9 +291,6 @@
     <t>Magia: Hechicería</t>
   </si>
   <si>
-    <t>Parpadeo (Estándar o Movimiento o Reacción, Instantáneo, 5 Foco)</t>
-  </si>
-  <si>
     <t>Descripciones de Rasgos y Poderes</t>
   </si>
   <si>
@@ -303,18 +300,6 @@
     <t>Tot. 10</t>
   </si>
   <si>
-    <t>Ataque de Ego vs Defensa de Agilidad a rango normal. En un éxito, mitad de daño y el objetivo esta Alentado. Si es Fantástico, el objetivo esta Restringido. En ambos casos, el efecto adicional dura hasta que se termine la Concentración.</t>
-  </si>
-  <si>
-    <t>Rayos de Balthaak (Estándar, Instantáneo + Concentración, 5 Foco)</t>
-  </si>
-  <si>
-    <t>Ataque de Ego vs Defensa de Agilidad a rango normal con Ventaja. En un éxito, daño normal. Si es Fantástico, doble daño y el objetivo esta Aturdido hasta que termine la Concentración.</t>
-  </si>
-  <si>
-    <t>Un aliado en rango gana Vida igual al Foco gastado - 5.</t>
-  </si>
-  <si>
     <t>Resiliencia + 1 x 20</t>
   </si>
   <si>
@@ -343,15 +328,6 @@
   </si>
   <si>
     <t>Chequeo de Ego. Detectas objetos, personas o lugares supernaturales dentro de 100 espacios por Grado. Sabes su localización y su estado general. Si un objeto, persona o lugar dentro del  rango se resiste o esta protegido, Chequeo de Ego vs Defensa de Ego (en caso de persona) o TN variable (en caso de objeto o lugar). En un éxito, lo detectas. Si es Fantástico, sabes la naturaleza exacta de la magia.</t>
-  </si>
-  <si>
-    <t>Te teletransportas hasta un numero de espacios igual a 10 x Grado, a un espacio que hayas visto.</t>
-  </si>
-  <si>
-    <t>Teletransporte (Estándar o Movimiento, Instantáneo, 10 Foco)</t>
-  </si>
-  <si>
-    <t>Cuando sos atacado. Te teletransportas hasta un numero de espacios igual a Grado, a un espacio que hayas visto. Si fuiste atacado y te mantuviste a rango o línea de visión, el ataque tiene Desventaja, sino el ataque falla.</t>
   </si>
   <si>
     <t>+5 Avances</t>
@@ -373,12 +349,6 @@
   </si>
   <si>
     <t>Primeros Auxilios (Estándar o Reacción, Concentración)</t>
-  </si>
-  <si>
-    <t>Cuando un aliado en alcance se vuelve Inconsciente. Una aliado en alcance pierde la condición de Inconsciente mientras mantienes la Concentración, pero solo puede tomar un Acción por ronda. Este poder también termina cuando la vida del aliado se vuelve mayor a 0.</t>
-  </si>
-  <si>
-    <t>Un aliado en alcance gana Vida igual al Foco gastado.</t>
   </si>
   <si>
     <t>+1 Ego  +1 Lógica</t>
@@ -399,7 +369,37 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Ataque de Ego vs Defensa de Agilidad a rango normal. En un éxito, mitad de daño y el objetivo esta Dañándose hasta que se termine la Concentración. Si es Fantástico, la condición de Dañándose hace 5 mas de daño de Vida. </t>
+    <t xml:space="preserve">Ataque de Ego vs Defensa de Agilidad a rango normal. En un éxito, mitad de daño de Aguante y el objetivo esta Dañándose hasta que se termine la Concentración. Si es Fantástico, la condición de Dañándose hace 5 mas de daño de Aguante. </t>
+  </si>
+  <si>
+    <t>Ataque de Ego vs Defensa de Agilidad a rango normal. En un éxito, mitad de daño de Aguante y el objetivo esta Alentado. Si es Fantástico, el objetivo esta Restringido. En ambos casos, el efecto adicional dura hasta que se termine la Concentración.</t>
+  </si>
+  <si>
+    <t>Teletransporte (Estándar y Movimiento, Instantáneo, 5 Foco)</t>
+  </si>
+  <si>
+    <t>Cuando un aliado en alcance se vuelve Inconsciente. Una aliado en alcance pierde la condición de Inconsciente mientras mantienes la Concentración, pero solo puede tomar una Acción por ronda. Este poder también termina cuando la vida del aliado se vuelve mayor a 0.</t>
+  </si>
+  <si>
+    <t>Ataque de Ego vs Defensa de Agilidad a rango normal. En un éxito, daño normal de Aguante. Si es Fantástico, doble daño y el objetivo esta Aturdido.</t>
+  </si>
+  <si>
+    <t>Te teletransportas hasta un numero de espacios igual a 10, a un espacio que hayas visto. Este movimiento cuenta como usar una Velocidad.</t>
+  </si>
+  <si>
+    <t>Parpadeo (Reacción o  Movimiento, Instantáneo)</t>
+  </si>
+  <si>
+    <t>Rayos de Balthaak (Estándar, Instantáneo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Un aliado en rango gana Aguante igual al Foco gastado + 5. </t>
+  </si>
+  <si>
+    <t>Un aliado en rango gana Aguante igual al Foco gastado.</t>
+  </si>
+  <si>
+    <t>Cuanto te atacan vs Defensas Físicas. Te teletransportas hasta un numero de espacios igual a 2, y a un espacio que hayas visto. Si ya no estas dentro del rango del ataque, o no puedes ser detectado, el enemigo atacante pierde su ataque.</t>
   </si>
 </sst>
 </file>
@@ -1383,7 +1383,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="263">
+  <cellXfs count="260">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1512,7 +1512,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1542,9 +1541,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="7" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1880,6 +1876,12 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="44" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1895,6 +1897,24 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -1919,39 +1939,6 @@
     <xf numFmtId="0" fontId="12" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2021,9 +2008,6 @@
     <xf numFmtId="0" fontId="12" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -2054,6 +2038,22 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="63" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="64" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2061,18 +2061,9 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2456,19 +2447,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="143" t="e" vm="1">
+      <c r="A1" s="141" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="B1" s="143"/>
-      <c r="C1" s="143"/>
-      <c r="D1" s="143"/>
-      <c r="E1" s="143"/>
+      <c r="B1" s="141"/>
+      <c r="C1" s="141"/>
+      <c r="D1" s="141"/>
+      <c r="E1" s="141"/>
       <c r="F1" s="30"/>
       <c r="G1" s="33" t="s">
         <v>37</v>
       </c>
-      <c r="H1" s="184"/>
-      <c r="I1" s="185"/>
+      <c r="H1" s="182"/>
+      <c r="I1" s="183"/>
       <c r="K1" s="48" t="s">
         <v>39</v>
       </c>
@@ -2476,53 +2467,53 @@
       <c r="N1" s="30"/>
     </row>
     <row r="2" spans="1:22" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="143"/>
-      <c r="B2" s="143"/>
-      <c r="C2" s="143"/>
-      <c r="D2" s="143"/>
-      <c r="E2" s="143"/>
+      <c r="A2" s="141"/>
+      <c r="B2" s="141"/>
+      <c r="C2" s="141"/>
+      <c r="D2" s="141"/>
+      <c r="E2" s="141"/>
       <c r="F2" s="30"/>
-      <c r="G2" s="186" t="s">
+      <c r="G2" s="184" t="s">
         <v>19</v>
       </c>
-      <c r="H2" s="188" t="s">
+      <c r="H2" s="186" t="s">
         <v>61</v>
       </c>
-      <c r="I2" s="189"/>
-      <c r="K2" s="84" t="s">
+      <c r="I2" s="187"/>
+      <c r="K2" s="82" t="s">
         <v>36</v>
       </c>
-      <c r="L2" s="85"/>
-      <c r="M2" s="86"/>
+      <c r="L2" s="83"/>
+      <c r="M2" s="84"/>
     </row>
     <row r="3" spans="1:22" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="143"/>
-      <c r="B3" s="143"/>
-      <c r="C3" s="143"/>
-      <c r="D3" s="143"/>
-      <c r="E3" s="143"/>
+      <c r="A3" s="141"/>
+      <c r="B3" s="141"/>
+      <c r="C3" s="141"/>
+      <c r="D3" s="141"/>
+      <c r="E3" s="141"/>
       <c r="F3" s="30"/>
-      <c r="G3" s="187"/>
-      <c r="H3" s="190"/>
-      <c r="I3" s="191"/>
-      <c r="K3" s="108" t="s">
+      <c r="G3" s="185"/>
+      <c r="H3" s="188"/>
+      <c r="I3" s="189"/>
+      <c r="K3" s="106" t="s">
         <v>41</v>
       </c>
-      <c r="L3" s="109"/>
-      <c r="M3" s="110"/>
+      <c r="L3" s="107"/>
+      <c r="M3" s="108"/>
     </row>
     <row r="4" spans="1:22" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="143"/>
-      <c r="B4" s="143"/>
-      <c r="C4" s="143"/>
-      <c r="D4" s="143"/>
-      <c r="E4" s="143"/>
+      <c r="A4" s="141"/>
+      <c r="B4" s="141"/>
+      <c r="C4" s="141"/>
+      <c r="D4" s="141"/>
+      <c r="E4" s="141"/>
       <c r="F4" s="30"/>
-      <c r="G4" s="186" t="s">
+      <c r="G4" s="184" t="s">
         <v>34</v>
       </c>
-      <c r="H4" s="188"/>
-      <c r="I4" s="189"/>
+      <c r="H4" s="186"/>
+      <c r="I4" s="187"/>
       <c r="K4" s="49" t="s">
         <v>42</v>
       </c>
@@ -2533,16 +2524,16 @@
       <c r="A5" s="58" t="s">
         <v>43</v>
       </c>
-      <c r="B5" s="97" t="s">
+      <c r="B5" s="95" t="s">
         <v>50</v>
       </c>
-      <c r="C5" s="97"/>
-      <c r="D5" s="98"/>
+      <c r="C5" s="95"/>
+      <c r="D5" s="96"/>
       <c r="E5" s="55"/>
       <c r="F5" s="30"/>
-      <c r="G5" s="187"/>
-      <c r="H5" s="190"/>
-      <c r="I5" s="191"/>
+      <c r="G5" s="185"/>
+      <c r="H5" s="188"/>
+      <c r="I5" s="189"/>
       <c r="K5" s="59" t="s">
         <v>58</v>
       </c>
@@ -2554,21 +2545,21 @@
       <c r="G6" s="33" t="s">
         <v>20</v>
       </c>
-      <c r="H6" s="184" t="s">
+      <c r="H6" s="182" t="s">
         <v>35</v>
       </c>
-      <c r="I6" s="185"/>
-      <c r="K6" s="192"/>
-      <c r="L6" s="193"/>
-      <c r="M6" s="194"/>
+      <c r="I6" s="183"/>
+      <c r="K6" s="190"/>
+      <c r="L6" s="191"/>
+      <c r="M6" s="192"/>
     </row>
     <row r="7" spans="1:22" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="140" t="s">
+      <c r="A7" s="138" t="s">
         <v>38</v>
       </c>
-      <c r="B7" s="141"/>
-      <c r="C7" s="141"/>
-      <c r="D7" s="142"/>
+      <c r="B7" s="139"/>
+      <c r="C7" s="139"/>
+      <c r="D7" s="140"/>
       <c r="E7" s="34" t="s">
         <v>46</v>
       </c>
@@ -2576,19 +2567,19 @@
       <c r="G7" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="H7" s="184"/>
-      <c r="I7" s="185"/>
-      <c r="K7" s="108"/>
-      <c r="L7" s="109"/>
-      <c r="M7" s="110"/>
+      <c r="H7" s="182"/>
+      <c r="I7" s="183"/>
+      <c r="K7" s="106"/>
+      <c r="L7" s="107"/>
+      <c r="M7" s="108"/>
       <c r="U7" s="30"/>
       <c r="V7" s="30"/>
     </row>
     <row r="8" spans="1:22" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="160"/>
-      <c r="B8" s="161"/>
-      <c r="C8" s="161"/>
-      <c r="D8" s="162"/>
+      <c r="A8" s="158"/>
+      <c r="B8" s="159"/>
+      <c r="C8" s="159"/>
+      <c r="D8" s="160"/>
       <c r="E8" s="35">
         <v>1</v>
       </c>
@@ -2596,13 +2587,13 @@
       <c r="G8" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="H8" s="184" t="s">
+      <c r="H8" s="182" t="s">
         <v>12</v>
       </c>
-      <c r="I8" s="185"/>
-      <c r="K8" s="108"/>
-      <c r="L8" s="109"/>
-      <c r="M8" s="110"/>
+      <c r="I8" s="183"/>
+      <c r="K8" s="106"/>
+      <c r="L8" s="107"/>
+      <c r="M8" s="108"/>
     </row>
     <row r="9" spans="1:22" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="30"/>
@@ -2611,62 +2602,62 @@
       <c r="D9" s="30"/>
       <c r="E9" s="30"/>
       <c r="F9" s="30"/>
-      <c r="K9" s="108"/>
-      <c r="L9" s="109"/>
-      <c r="M9" s="110"/>
+      <c r="K9" s="106"/>
+      <c r="L9" s="107"/>
+      <c r="M9" s="108"/>
     </row>
     <row r="10" spans="1:22" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="172" t="s">
-        <v>71</v>
-      </c>
-      <c r="B10" s="173"/>
-      <c r="C10" s="173"/>
-      <c r="D10" s="174"/>
-      <c r="E10" s="154" t="s">
+      <c r="A10" s="170" t="s">
+        <v>66</v>
+      </c>
+      <c r="B10" s="171"/>
+      <c r="C10" s="171"/>
+      <c r="D10" s="172"/>
+      <c r="E10" s="152" t="s">
         <v>31</v>
       </c>
       <c r="F10" s="30"/>
-      <c r="G10" s="87" t="s">
+      <c r="G10" s="85" t="s">
         <v>59</v>
       </c>
-      <c r="H10" s="88"/>
-      <c r="I10" s="89"/>
-      <c r="K10" s="195"/>
-      <c r="L10" s="196"/>
-      <c r="M10" s="197"/>
+      <c r="H10" s="86"/>
+      <c r="I10" s="87"/>
+      <c r="K10" s="193"/>
+      <c r="L10" s="194"/>
+      <c r="M10" s="195"/>
     </row>
     <row r="11" spans="1:22" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="75" t="s">
-        <v>70</v>
-      </c>
-      <c r="B11" s="76"/>
-      <c r="C11" s="76"/>
-      <c r="D11" s="77"/>
-      <c r="E11" s="155"/>
+      <c r="A11" s="73" t="s">
+        <v>65</v>
+      </c>
+      <c r="B11" s="74"/>
+      <c r="C11" s="74"/>
+      <c r="D11" s="75"/>
+      <c r="E11" s="153"/>
       <c r="F11" s="30"/>
-      <c r="G11" s="178"/>
-      <c r="H11" s="179"/>
-      <c r="I11" s="180"/>
-      <c r="K11" s="175"/>
-      <c r="L11" s="176"/>
-      <c r="M11" s="177"/>
+      <c r="G11" s="176"/>
+      <c r="H11" s="177"/>
+      <c r="I11" s="178"/>
+      <c r="K11" s="173"/>
+      <c r="L11" s="174"/>
+      <c r="M11" s="175"/>
     </row>
     <row r="12" spans="1:22" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="158"/>
-      <c r="B12" s="159"/>
-      <c r="C12" s="71" t="str">
+      <c r="A12" s="156"/>
+      <c r="B12" s="157"/>
+      <c r="C12" s="70" t="str">
         <f>_xlfn.CONCAT("/",IF(A32=0,20,20 + A32*IF(Modifiers!O5,Modifiers!O5,20)) + Modifiers!N5)</f>
-        <v>/20</v>
-      </c>
-      <c r="D12" s="72"/>
+        <v>/40</v>
+      </c>
+      <c r="D12" s="71"/>
       <c r="E12" s="31"/>
       <c r="F12" s="30"/>
-      <c r="G12" s="81"/>
-      <c r="H12" s="82"/>
-      <c r="I12" s="83"/>
-      <c r="K12" s="108"/>
-      <c r="L12" s="109"/>
-      <c r="M12" s="110"/>
+      <c r="G12" s="79"/>
+      <c r="H12" s="80"/>
+      <c r="I12" s="81"/>
+      <c r="K12" s="106"/>
+      <c r="L12" s="107"/>
+      <c r="M12" s="108"/>
     </row>
     <row r="13" spans="1:22" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="30"/>
@@ -2675,63 +2666,63 @@
       <c r="D13" s="30"/>
       <c r="E13" s="30"/>
       <c r="F13" s="30"/>
-      <c r="G13" s="81"/>
-      <c r="H13" s="82"/>
-      <c r="I13" s="83"/>
-      <c r="K13" s="108"/>
-      <c r="L13" s="109"/>
-      <c r="M13" s="110"/>
+      <c r="G13" s="79"/>
+      <c r="H13" s="80"/>
+      <c r="I13" s="81"/>
+      <c r="K13" s="106"/>
+      <c r="L13" s="107"/>
+      <c r="M13" s="108"/>
     </row>
     <row r="14" spans="1:22" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="66" t="s">
-        <v>72</v>
-      </c>
-      <c r="B14" s="68"/>
-      <c r="C14" s="68"/>
-      <c r="D14" s="69"/>
-      <c r="E14" s="154" t="s">
+      <c r="A14" s="65" t="s">
+        <v>67</v>
+      </c>
+      <c r="B14" s="67"/>
+      <c r="C14" s="67"/>
+      <c r="D14" s="68"/>
+      <c r="E14" s="152" t="s">
         <v>31</v>
       </c>
       <c r="F14" s="30"/>
-      <c r="G14" s="81"/>
-      <c r="H14" s="82"/>
-      <c r="I14" s="83"/>
-      <c r="K14" s="108"/>
-      <c r="L14" s="109"/>
-      <c r="M14" s="110"/>
+      <c r="G14" s="79"/>
+      <c r="H14" s="80"/>
+      <c r="I14" s="81"/>
+      <c r="K14" s="106"/>
+      <c r="L14" s="107"/>
+      <c r="M14" s="108"/>
     </row>
     <row r="15" spans="1:22" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="75" t="s">
-        <v>76</v>
-      </c>
-      <c r="B15" s="76"/>
-      <c r="C15" s="76"/>
-      <c r="D15" s="77"/>
-      <c r="E15" s="155"/>
+      <c r="A15" s="73" t="s">
+        <v>71</v>
+      </c>
+      <c r="B15" s="74"/>
+      <c r="C15" s="74"/>
+      <c r="D15" s="75"/>
+      <c r="E15" s="153"/>
       <c r="F15" s="30"/>
-      <c r="G15" s="181"/>
-      <c r="H15" s="182"/>
-      <c r="I15" s="183"/>
-      <c r="K15" s="108"/>
-      <c r="L15" s="109"/>
-      <c r="M15" s="110"/>
+      <c r="G15" s="179"/>
+      <c r="H15" s="180"/>
+      <c r="I15" s="181"/>
+      <c r="K15" s="106"/>
+      <c r="L15" s="107"/>
+      <c r="M15" s="108"/>
     </row>
     <row r="16" spans="1:22" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="158"/>
-      <c r="B16" s="159"/>
-      <c r="C16" s="71" t="str">
+      <c r="A16" s="156"/>
+      <c r="B16" s="157"/>
+      <c r="C16" s="70" t="str">
         <f>_xlfn.CONCAT("/",IF(A34=0,20,20 + A34 * IF(Modifiers!O6,Modifiers!O6,20)) + Modifiers!N6)</f>
         <v>/80</v>
       </c>
-      <c r="D16" s="72"/>
+      <c r="D16" s="71"/>
       <c r="E16" s="31"/>
       <c r="F16" s="30"/>
-      <c r="G16" s="81"/>
-      <c r="H16" s="82"/>
-      <c r="I16" s="83"/>
-      <c r="K16" s="108"/>
-      <c r="L16" s="109"/>
-      <c r="M16" s="110"/>
+      <c r="G16" s="79"/>
+      <c r="H16" s="80"/>
+      <c r="I16" s="81"/>
+      <c r="K16" s="106"/>
+      <c r="L16" s="107"/>
+      <c r="M16" s="108"/>
     </row>
     <row r="17" spans="1:14" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="30"/>
@@ -2740,90 +2731,90 @@
       <c r="D17" s="30"/>
       <c r="E17" s="30"/>
       <c r="F17" s="30"/>
-      <c r="G17" s="81"/>
-      <c r="H17" s="82"/>
-      <c r="I17" s="83"/>
-      <c r="K17" s="108"/>
-      <c r="L17" s="109"/>
-      <c r="M17" s="110"/>
+      <c r="G17" s="79"/>
+      <c r="H17" s="80"/>
+      <c r="I17" s="81"/>
+      <c r="K17" s="106"/>
+      <c r="L17" s="107"/>
+      <c r="M17" s="108"/>
     </row>
     <row r="18" spans="1:14" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="67" t="s">
-        <v>75</v>
-      </c>
-      <c r="B18" s="68"/>
-      <c r="C18" s="70"/>
-      <c r="D18" s="156"/>
-      <c r="E18" s="154" t="s">
+      <c r="A18" s="66" t="s">
+        <v>70</v>
+      </c>
+      <c r="B18" s="67"/>
+      <c r="C18" s="69"/>
+      <c r="D18" s="154"/>
+      <c r="E18" s="152" t="s">
         <v>32</v>
       </c>
       <c r="F18" s="30"/>
-      <c r="G18" s="102"/>
-      <c r="H18" s="103"/>
-      <c r="I18" s="104"/>
-      <c r="K18" s="108"/>
-      <c r="L18" s="109"/>
-      <c r="M18" s="110"/>
+      <c r="G18" s="100"/>
+      <c r="H18" s="101"/>
+      <c r="I18" s="102"/>
+      <c r="K18" s="106"/>
+      <c r="L18" s="107"/>
+      <c r="M18" s="108"/>
     </row>
     <row r="19" spans="1:14" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="78" t="s">
+      <c r="A19" s="76" t="s">
         <v>46</v>
       </c>
-      <c r="B19" s="79"/>
-      <c r="C19" s="80"/>
-      <c r="D19" s="157"/>
-      <c r="E19" s="155"/>
+      <c r="B19" s="77"/>
+      <c r="C19" s="78"/>
+      <c r="D19" s="155"/>
+      <c r="E19" s="153"/>
       <c r="F19" s="30"/>
-      <c r="G19" s="99" t="s">
+      <c r="G19" s="97" t="s">
         <v>60</v>
       </c>
-      <c r="H19" s="100"/>
-      <c r="I19" s="101"/>
-      <c r="K19" s="108"/>
-      <c r="L19" s="109"/>
-      <c r="M19" s="110"/>
+      <c r="H19" s="98"/>
+      <c r="I19" s="99"/>
+      <c r="K19" s="106"/>
+      <c r="L19" s="107"/>
+      <c r="M19" s="108"/>
     </row>
     <row r="20" spans="1:14" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="169" t="s">
+      <c r="A20" s="167" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="170"/>
-      <c r="C20" s="170"/>
-      <c r="D20" s="171"/>
+      <c r="B20" s="168"/>
+      <c r="C20" s="168"/>
+      <c r="D20" s="169"/>
       <c r="E20" s="32" t="str">
         <f>_xlfn.CONCAT("+",IF(Modifiers!K6="Edge",_xlfn.CONCAT(A34,"E"),A34))</f>
         <v>+3</v>
       </c>
       <c r="F20" s="30"/>
-      <c r="G20" s="81"/>
-      <c r="H20" s="82"/>
-      <c r="I20" s="83"/>
-      <c r="K20" s="108"/>
-      <c r="L20" s="109"/>
-      <c r="M20" s="110"/>
+      <c r="G20" s="79"/>
+      <c r="H20" s="80"/>
+      <c r="I20" s="81"/>
+      <c r="K20" s="106"/>
+      <c r="L20" s="107"/>
+      <c r="M20" s="108"/>
     </row>
     <row r="21" spans="1:14" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="118" t="s">
+      <c r="A21" s="116" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="119"/>
-      <c r="C21" s="119"/>
-      <c r="D21" s="119"/>
-      <c r="E21" s="120"/>
+      <c r="B21" s="117"/>
+      <c r="C21" s="117"/>
+      <c r="D21" s="117"/>
+      <c r="E21" s="118"/>
       <c r="F21" s="30"/>
-      <c r="G21" s="105"/>
-      <c r="H21" s="106"/>
-      <c r="I21" s="107"/>
-      <c r="K21" s="113"/>
-      <c r="L21" s="114"/>
-      <c r="M21" s="115"/>
+      <c r="G21" s="103"/>
+      <c r="H21" s="104"/>
+      <c r="I21" s="105"/>
+      <c r="K21" s="111"/>
+      <c r="L21" s="112"/>
+      <c r="M21" s="113"/>
     </row>
     <row r="22" spans="1:14" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="118"/>
-      <c r="B22" s="119"/>
-      <c r="C22" s="119"/>
-      <c r="D22" s="119"/>
-      <c r="E22" s="165"/>
+      <c r="A22" s="116"/>
+      <c r="B22" s="117"/>
+      <c r="C22" s="117"/>
+      <c r="D22" s="117"/>
+      <c r="E22" s="163"/>
       <c r="F22" s="30"/>
       <c r="J22" s="30"/>
       <c r="K22" s="30"/>
@@ -2832,11 +2823,11 @@
       <c r="N22" s="30"/>
     </row>
     <row r="23" spans="1:14" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="163"/>
-      <c r="B23" s="164"/>
-      <c r="C23" s="161"/>
-      <c r="D23" s="161"/>
-      <c r="E23" s="162"/>
+      <c r="A23" s="161"/>
+      <c r="B23" s="162"/>
+      <c r="C23" s="159"/>
+      <c r="D23" s="159"/>
+      <c r="E23" s="160"/>
       <c r="F23" s="30"/>
       <c r="G23" s="43" t="s">
         <v>18</v>
@@ -2861,7 +2852,7 @@
       </c>
       <c r="H24" s="45"/>
       <c r="I24" s="39" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="J24" s="39"/>
       <c r="K24" s="39"/>
@@ -2869,13 +2860,13 @@
       <c r="M24" s="40"/>
     </row>
     <row r="25" spans="1:14" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="166" t="s">
+      <c r="A25" s="164" t="s">
         <v>25</v>
       </c>
-      <c r="B25" s="167"/>
-      <c r="C25" s="167"/>
-      <c r="D25" s="167"/>
-      <c r="E25" s="168"/>
+      <c r="B25" s="165"/>
+      <c r="C25" s="165"/>
+      <c r="D25" s="165"/>
+      <c r="E25" s="166"/>
       <c r="F25" s="30"/>
       <c r="G25" s="46"/>
       <c r="H25" s="47"/>
@@ -2886,15 +2877,15 @@
       <c r="M25" s="37"/>
     </row>
     <row r="26" spans="1:14" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="148" t="s">
+      <c r="A26" s="146" t="s">
         <v>26</v>
       </c>
-      <c r="B26" s="149"/>
-      <c r="C26" s="149"/>
-      <c r="D26" s="149" t="s">
+      <c r="B26" s="147"/>
+      <c r="C26" s="147"/>
+      <c r="D26" s="147" t="s">
         <v>27</v>
       </c>
-      <c r="E26" s="152"/>
+      <c r="E26" s="150"/>
       <c r="F26" s="30"/>
       <c r="G26" s="46"/>
       <c r="H26" s="47"/>
@@ -2905,72 +2896,72 @@
       <c r="M26" s="37"/>
     </row>
     <row r="27" spans="1:14" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="150"/>
-      <c r="B27" s="151"/>
-      <c r="C27" s="151"/>
-      <c r="D27" s="151"/>
-      <c r="E27" s="153"/>
+      <c r="A27" s="148"/>
+      <c r="B27" s="149"/>
+      <c r="C27" s="149"/>
+      <c r="D27" s="149"/>
+      <c r="E27" s="151"/>
       <c r="F27" s="30"/>
       <c r="G27" s="46" t="s">
         <v>61</v>
       </c>
       <c r="H27" s="47"/>
-      <c r="I27" s="111" t="s">
-        <v>78</v>
-      </c>
-      <c r="J27" s="111"/>
-      <c r="K27" s="111"/>
-      <c r="L27" s="111"/>
-      <c r="M27" s="112"/>
+      <c r="I27" s="109" t="s">
+        <v>73</v>
+      </c>
+      <c r="J27" s="109"/>
+      <c r="K27" s="109"/>
+      <c r="L27" s="109"/>
+      <c r="M27" s="110"/>
     </row>
     <row r="28" spans="1:14" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="145">
+      <c r="A28" s="143">
         <v>0</v>
       </c>
-      <c r="B28" s="146"/>
-      <c r="C28" s="147"/>
-      <c r="D28" s="136">
+      <c r="B28" s="144"/>
+      <c r="C28" s="145"/>
+      <c r="D28" s="134">
         <f xml:space="preserve"> 10 + A28 + Modifiers!B3</f>
         <v>10</v>
       </c>
-      <c r="E28" s="137"/>
+      <c r="E28" s="135"/>
       <c r="F28" s="30"/>
       <c r="G28" s="46"/>
       <c r="H28" s="47"/>
-      <c r="I28" s="111"/>
-      <c r="J28" s="111"/>
-      <c r="K28" s="111"/>
-      <c r="L28" s="111"/>
-      <c r="M28" s="112"/>
+      <c r="I28" s="109"/>
+      <c r="J28" s="109"/>
+      <c r="K28" s="109"/>
+      <c r="L28" s="109"/>
+      <c r="M28" s="110"/>
     </row>
     <row r="29" spans="1:14" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="121" t="s">
-        <v>64</v>
-      </c>
-      <c r="B29" s="122"/>
-      <c r="C29" s="123"/>
-      <c r="D29" s="138"/>
-      <c r="E29" s="139"/>
+      <c r="A29" s="119" t="s">
+        <v>63</v>
+      </c>
+      <c r="B29" s="120"/>
+      <c r="C29" s="121"/>
+      <c r="D29" s="136"/>
+      <c r="E29" s="137"/>
       <c r="F29" s="30"/>
       <c r="G29" s="46"/>
       <c r="H29" s="47"/>
-      <c r="I29" s="111"/>
-      <c r="J29" s="111"/>
-      <c r="K29" s="111"/>
-      <c r="L29" s="111"/>
-      <c r="M29" s="112"/>
+      <c r="I29" s="109"/>
+      <c r="J29" s="109"/>
+      <c r="K29" s="109"/>
+      <c r="L29" s="109"/>
+      <c r="M29" s="110"/>
     </row>
     <row r="30" spans="1:14" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="145">
+      <c r="A30" s="143">
         <v>1</v>
       </c>
-      <c r="B30" s="146"/>
-      <c r="C30" s="147"/>
-      <c r="D30" s="136">
+      <c r="B30" s="144"/>
+      <c r="C30" s="145"/>
+      <c r="D30" s="134">
         <f>IF(Modifiers!C4,Modifiers!C4,10 + A30 + Modifiers!B4)</f>
         <v>11</v>
       </c>
-      <c r="E30" s="137"/>
+      <c r="E30" s="135"/>
       <c r="F30" s="30"/>
       <c r="G30" s="46"/>
       <c r="H30" s="47"/>
@@ -2981,13 +2972,13 @@
       <c r="M30" s="37"/>
     </row>
     <row r="31" spans="1:14" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="121" t="s">
+      <c r="A31" s="119" t="s">
         <v>28</v>
       </c>
-      <c r="B31" s="122"/>
-      <c r="C31" s="123"/>
-      <c r="D31" s="138"/>
-      <c r="E31" s="139"/>
+      <c r="B31" s="120"/>
+      <c r="C31" s="121"/>
+      <c r="D31" s="136"/>
+      <c r="E31" s="137"/>
       <c r="F31" s="30"/>
       <c r="G31" s="46"/>
       <c r="H31" s="47"/>
@@ -2998,16 +2989,16 @@
       <c r="M31" s="37"/>
     </row>
     <row r="32" spans="1:14" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="145">
-        <v>0</v>
-      </c>
-      <c r="B32" s="146"/>
-      <c r="C32" s="147"/>
-      <c r="D32" s="136">
+      <c r="A32" s="143">
+        <v>1</v>
+      </c>
+      <c r="B32" s="144"/>
+      <c r="C32" s="145"/>
+      <c r="D32" s="134">
         <f xml:space="preserve"> 10 + A32 + Modifiers!B5</f>
-        <v>10</v>
-      </c>
-      <c r="E32" s="137"/>
+        <v>11</v>
+      </c>
+      <c r="E32" s="135"/>
       <c r="F32" s="30"/>
       <c r="G32" s="46"/>
       <c r="H32" s="47"/>
@@ -3018,13 +3009,13 @@
       <c r="M32" s="37"/>
     </row>
     <row r="33" spans="1:14" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="121" t="s">
+      <c r="A33" s="119" t="s">
         <v>30</v>
       </c>
-      <c r="B33" s="122"/>
-      <c r="C33" s="123"/>
-      <c r="D33" s="138"/>
-      <c r="E33" s="139"/>
+      <c r="B33" s="120"/>
+      <c r="C33" s="121"/>
+      <c r="D33" s="136"/>
+      <c r="E33" s="137"/>
       <c r="F33" s="30"/>
       <c r="G33" s="46"/>
       <c r="H33" s="47"/>
@@ -3035,16 +3026,16 @@
       <c r="M33" s="37"/>
     </row>
     <row r="34" spans="1:14" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="145">
+      <c r="A34" s="143">
         <v>3</v>
       </c>
-      <c r="B34" s="146"/>
-      <c r="C34" s="147"/>
-      <c r="D34" s="136">
+      <c r="B34" s="144"/>
+      <c r="C34" s="145"/>
+      <c r="D34" s="134">
         <f xml:space="preserve"> 10 + A34 + Modifiers!B6</f>
         <v>13</v>
       </c>
-      <c r="E34" s="137"/>
+      <c r="E34" s="135"/>
       <c r="F34" s="30"/>
       <c r="G34" s="46"/>
       <c r="H34" s="47"/>
@@ -3055,13 +3046,13 @@
       <c r="M34" s="37"/>
     </row>
     <row r="35" spans="1:14" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="121" t="s">
+      <c r="A35" s="119" t="s">
         <v>29</v>
       </c>
-      <c r="B35" s="122"/>
-      <c r="C35" s="123"/>
-      <c r="D35" s="138"/>
-      <c r="E35" s="139"/>
+      <c r="B35" s="120"/>
+      <c r="C35" s="121"/>
+      <c r="D35" s="136"/>
+      <c r="E35" s="137"/>
       <c r="F35" s="30"/>
       <c r="G35" s="46"/>
       <c r="H35" s="47"/>
@@ -3072,16 +3063,16 @@
       <c r="M35" s="37"/>
     </row>
     <row r="36" spans="1:14" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="145">
+      <c r="A36" s="143">
         <v>1</v>
       </c>
-      <c r="B36" s="146"/>
-      <c r="C36" s="147"/>
-      <c r="D36" s="136">
+      <c r="B36" s="144"/>
+      <c r="C36" s="145"/>
+      <c r="D36" s="134">
         <f xml:space="preserve"> 10 + A36 + Modifiers!B7</f>
         <v>11</v>
       </c>
-      <c r="E36" s="137"/>
+      <c r="E36" s="135"/>
       <c r="F36" s="30"/>
       <c r="G36" s="46"/>
       <c r="H36" s="47"/>
@@ -3092,13 +3083,13 @@
       <c r="M36" s="37"/>
     </row>
     <row r="37" spans="1:14" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="121" t="s">
+      <c r="A37" s="119" t="s">
         <v>5</v>
       </c>
-      <c r="B37" s="122"/>
-      <c r="C37" s="123"/>
-      <c r="D37" s="138"/>
-      <c r="E37" s="139"/>
+      <c r="B37" s="120"/>
+      <c r="C37" s="121"/>
+      <c r="D37" s="136"/>
+      <c r="E37" s="137"/>
       <c r="F37" s="30"/>
       <c r="G37" s="46"/>
       <c r="H37" s="47"/>
@@ -3109,16 +3100,16 @@
       <c r="M37" s="37"/>
     </row>
     <row r="38" spans="1:14" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="136">
-        <v>1</v>
-      </c>
-      <c r="B38" s="144"/>
-      <c r="C38" s="137"/>
-      <c r="D38" s="136">
+      <c r="A38" s="134">
+        <v>0</v>
+      </c>
+      <c r="B38" s="142"/>
+      <c r="C38" s="135"/>
+      <c r="D38" s="134">
         <f xml:space="preserve"> 10 + A38 + Modifiers!B8</f>
-        <v>11</v>
-      </c>
-      <c r="E38" s="137"/>
+        <v>10</v>
+      </c>
+      <c r="E38" s="135"/>
       <c r="F38" s="30"/>
       <c r="G38" s="46"/>
       <c r="H38" s="47"/>
@@ -3129,13 +3120,13 @@
       <c r="M38" s="37"/>
     </row>
     <row r="39" spans="1:14" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="121" t="s">
+      <c r="A39" s="119" t="s">
         <v>33</v>
       </c>
-      <c r="B39" s="122"/>
-      <c r="C39" s="123"/>
-      <c r="D39" s="138"/>
-      <c r="E39" s="139"/>
+      <c r="B39" s="120"/>
+      <c r="C39" s="121"/>
+      <c r="D39" s="136"/>
+      <c r="E39" s="137"/>
       <c r="F39" s="30"/>
       <c r="G39" s="46"/>
       <c r="H39" s="47"/>
@@ -3152,22 +3143,22 @@
       <c r="D40" s="30"/>
       <c r="E40" s="30"/>
       <c r="F40" s="30"/>
-      <c r="G40" s="94"/>
-      <c r="H40" s="95"/>
-      <c r="I40" s="95"/>
-      <c r="J40" s="95"/>
-      <c r="K40" s="95"/>
-      <c r="L40" s="95"/>
-      <c r="M40" s="96"/>
+      <c r="G40" s="92"/>
+      <c r="H40" s="93"/>
+      <c r="I40" s="93"/>
+      <c r="J40" s="93"/>
+      <c r="K40" s="93"/>
+      <c r="L40" s="93"/>
+      <c r="M40" s="94"/>
     </row>
     <row r="41" spans="1:14" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="132" t="s">
+      <c r="A41" s="130" t="s">
         <v>24</v>
       </c>
-      <c r="B41" s="133"/>
-      <c r="C41" s="133"/>
-      <c r="D41" s="133"/>
-      <c r="E41" s="134"/>
+      <c r="B41" s="131"/>
+      <c r="C41" s="131"/>
+      <c r="D41" s="131"/>
+      <c r="E41" s="132"/>
       <c r="F41" s="30"/>
       <c r="G41" s="30"/>
       <c r="H41" s="30"/>
@@ -3178,20 +3169,20 @@
       <c r="M41" s="30"/>
     </row>
     <row r="42" spans="1:14" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="124" t="s">
-        <v>64</v>
-      </c>
-      <c r="B42" s="116" t="e" vm="2">
+      <c r="A42" s="122" t="s">
+        <v>63</v>
+      </c>
+      <c r="B42" s="114" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
-      <c r="C42" s="126" t="str">
+      <c r="C42" s="124" t="str">
         <f>_xlfn.CONCAT("X ",IF(Modifiers!G3,Modifiers!G3,$E$8 + Modifiers!F3))</f>
         <v>X 1</v>
       </c>
-      <c r="D42" s="135" t="s">
+      <c r="D42" s="133" t="s">
         <v>7</v>
       </c>
-      <c r="E42" s="130">
+      <c r="E42" s="128">
         <f>A28</f>
         <v>0</v>
       </c>
@@ -3207,11 +3198,11 @@
       <c r="M42" s="30"/>
     </row>
     <row r="43" spans="1:14" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="124"/>
-      <c r="B43" s="116"/>
-      <c r="C43" s="126"/>
-      <c r="D43" s="128"/>
-      <c r="E43" s="130"/>
+      <c r="A43" s="122"/>
+      <c r="B43" s="114"/>
+      <c r="C43" s="124"/>
+      <c r="D43" s="126"/>
+      <c r="E43" s="128"/>
       <c r="F43" s="30"/>
       <c r="G43" s="50"/>
       <c r="H43" s="51"/>
@@ -3222,20 +3213,20 @@
       <c r="M43" s="52"/>
     </row>
     <row r="44" spans="1:14" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="124" t="s">
+      <c r="A44" s="122" t="s">
         <v>28</v>
       </c>
-      <c r="B44" s="116" t="e" vm="2">
+      <c r="B44" s="114" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
-      <c r="C44" s="126" t="str">
+      <c r="C44" s="124" t="str">
         <f>_xlfn.CONCAT("X ",IF(Modifiers!G5,Modifiers!G5,$E$8 + Modifiers!F5))</f>
         <v>X 1</v>
       </c>
-      <c r="D44" s="128" t="s">
+      <c r="D44" s="126" t="s">
         <v>7</v>
       </c>
-      <c r="E44" s="130">
+      <c r="E44" s="128">
         <f>A30</f>
         <v>1</v>
       </c>
@@ -3249,11 +3240,11 @@
       <c r="M44" s="53"/>
     </row>
     <row r="45" spans="1:14" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="124"/>
-      <c r="B45" s="116"/>
-      <c r="C45" s="126"/>
-      <c r="D45" s="128"/>
-      <c r="E45" s="130"/>
+      <c r="A45" s="122"/>
+      <c r="B45" s="114"/>
+      <c r="C45" s="124"/>
+      <c r="D45" s="126"/>
+      <c r="E45" s="128"/>
       <c r="F45" s="30"/>
       <c r="G45" s="38"/>
       <c r="H45" s="36"/>
@@ -3265,20 +3256,20 @@
       <c r="N45" s="30"/>
     </row>
     <row r="46" spans="1:14" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="124" t="s">
+      <c r="A46" s="122" t="s">
         <v>5</v>
       </c>
-      <c r="B46" s="116" t="e" vm="2">
+      <c r="B46" s="114" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
-      <c r="C46" s="126" t="str">
+      <c r="C46" s="124" t="str">
         <f>_xlfn.CONCAT("X ",IF(Modifiers!G7,Modifiers!G7,$E$8 + Modifiers!F7))</f>
         <v>X 1</v>
       </c>
-      <c r="D46" s="128" t="s">
+      <c r="D46" s="126" t="s">
         <v>7</v>
       </c>
-      <c r="E46" s="130">
+      <c r="E46" s="128">
         <f>A36</f>
         <v>1</v>
       </c>
@@ -3293,61 +3284,61 @@
       <c r="N46" s="30"/>
     </row>
     <row r="47" spans="1:14" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="124"/>
-      <c r="B47" s="116"/>
-      <c r="C47" s="126"/>
-      <c r="D47" s="128"/>
-      <c r="E47" s="130"/>
+      <c r="A47" s="122"/>
+      <c r="B47" s="114"/>
+      <c r="C47" s="124"/>
+      <c r="D47" s="126"/>
+      <c r="E47" s="128"/>
       <c r="F47" s="30"/>
-      <c r="G47" s="81"/>
-      <c r="H47" s="82"/>
-      <c r="I47" s="82"/>
-      <c r="J47" s="82"/>
-      <c r="K47" s="82"/>
-      <c r="L47" s="82"/>
-      <c r="M47" s="83"/>
+      <c r="G47" s="79"/>
+      <c r="H47" s="80"/>
+      <c r="I47" s="80"/>
+      <c r="J47" s="80"/>
+      <c r="K47" s="80"/>
+      <c r="L47" s="80"/>
+      <c r="M47" s="81"/>
     </row>
     <row r="48" spans="1:14" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="124" t="s">
+      <c r="A48" s="122" t="s">
         <v>33</v>
       </c>
-      <c r="B48" s="116" t="e" vm="2">
+      <c r="B48" s="114" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
-      <c r="C48" s="126" t="str">
+      <c r="C48" s="124" t="str">
         <f>_xlfn.CONCAT("X ",IF(Modifiers!G9,Modifiers!G9,$E$8 + Modifiers!F9))</f>
         <v>X 1</v>
       </c>
-      <c r="D48" s="128" t="s">
+      <c r="D48" s="126" t="s">
         <v>7</v>
       </c>
-      <c r="E48" s="130">
+      <c r="E48" s="128">
         <f>A38</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F48" s="30"/>
-      <c r="G48" s="81"/>
-      <c r="H48" s="82"/>
-      <c r="I48" s="82"/>
-      <c r="J48" s="82"/>
-      <c r="K48" s="82"/>
-      <c r="L48" s="82"/>
-      <c r="M48" s="83"/>
+      <c r="G48" s="79"/>
+      <c r="H48" s="80"/>
+      <c r="I48" s="80"/>
+      <c r="J48" s="80"/>
+      <c r="K48" s="80"/>
+      <c r="L48" s="80"/>
+      <c r="M48" s="81"/>
     </row>
     <row r="49" spans="1:13" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="125"/>
-      <c r="B49" s="117"/>
-      <c r="C49" s="127"/>
-      <c r="D49" s="129"/>
-      <c r="E49" s="131"/>
+      <c r="A49" s="123"/>
+      <c r="B49" s="115"/>
+      <c r="C49" s="125"/>
+      <c r="D49" s="127"/>
+      <c r="E49" s="129"/>
       <c r="F49" s="30"/>
-      <c r="G49" s="81"/>
-      <c r="H49" s="82"/>
-      <c r="I49" s="82"/>
-      <c r="J49" s="82"/>
-      <c r="K49" s="82"/>
-      <c r="L49" s="82"/>
-      <c r="M49" s="83"/>
+      <c r="G49" s="79"/>
+      <c r="H49" s="80"/>
+      <c r="I49" s="80"/>
+      <c r="J49" s="80"/>
+      <c r="K49" s="80"/>
+      <c r="L49" s="80"/>
+      <c r="M49" s="81"/>
     </row>
     <row r="50" spans="1:13" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="30"/>
@@ -3365,13 +3356,13 @@
       <c r="M50" s="37"/>
     </row>
     <row r="51" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="67" t="s">
-        <v>73</v>
-      </c>
-      <c r="B51" s="68"/>
-      <c r="C51" s="68"/>
-      <c r="D51" s="68"/>
-      <c r="E51" s="69"/>
+      <c r="A51" s="66" t="s">
+        <v>68</v>
+      </c>
+      <c r="B51" s="67"/>
+      <c r="C51" s="67"/>
+      <c r="D51" s="67"/>
+      <c r="E51" s="68"/>
       <c r="F51" s="30"/>
       <c r="G51" s="46"/>
       <c r="H51" s="47"/>
@@ -3382,13 +3373,13 @@
       <c r="M51" s="37"/>
     </row>
     <row r="52" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="75" t="s">
-        <v>74</v>
-      </c>
-      <c r="B52" s="76"/>
-      <c r="C52" s="76"/>
-      <c r="D52" s="76"/>
-      <c r="E52" s="77"/>
+      <c r="A52" s="73" t="s">
+        <v>69</v>
+      </c>
+      <c r="B52" s="74"/>
+      <c r="C52" s="74"/>
+      <c r="D52" s="74"/>
+      <c r="E52" s="75"/>
       <c r="F52" s="30"/>
       <c r="G52" s="46"/>
       <c r="H52" s="47"/>
@@ -3399,23 +3390,23 @@
       <c r="M52" s="37"/>
     </row>
     <row r="53" spans="1:13" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="90"/>
-      <c r="B53" s="91"/>
-      <c r="C53" s="92" t="s">
+      <c r="A53" s="88"/>
+      <c r="B53" s="89"/>
+      <c r="C53" s="90" t="s">
         <v>44</v>
       </c>
-      <c r="D53" s="93"/>
+      <c r="D53" s="91"/>
       <c r="E53" s="54" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F53" s="30"/>
-      <c r="G53" s="94"/>
-      <c r="H53" s="95"/>
-      <c r="I53" s="95"/>
-      <c r="J53" s="95"/>
-      <c r="K53" s="95"/>
-      <c r="L53" s="95"/>
-      <c r="M53" s="96"/>
+      <c r="G53" s="92"/>
+      <c r="H53" s="93"/>
+      <c r="I53" s="93"/>
+      <c r="J53" s="93"/>
+      <c r="K53" s="93"/>
+      <c r="L53" s="93"/>
+      <c r="M53" s="94"/>
     </row>
     <row r="54" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F54" s="30"/>
@@ -3546,118 +3537,118 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="203" t="s">
-        <v>63</v>
-      </c>
-      <c r="B1" s="204"/>
-      <c r="C1" s="204"/>
-      <c r="D1" s="205"/>
+      <c r="A1" s="209" t="s">
+        <v>62</v>
+      </c>
+      <c r="B1" s="210"/>
+      <c r="C1" s="210"/>
+      <c r="D1" s="211"/>
     </row>
     <row r="2" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="208"/>
-      <c r="B2" s="209"/>
-      <c r="C2" s="209"/>
-      <c r="D2" s="209"/>
-      <c r="E2" s="209"/>
-      <c r="F2" s="209"/>
-      <c r="G2" s="209"/>
-      <c r="H2" s="209"/>
-      <c r="I2" s="210"/>
+      <c r="A2" s="214"/>
+      <c r="B2" s="215"/>
+      <c r="C2" s="215"/>
+      <c r="D2" s="215"/>
+      <c r="E2" s="215"/>
+      <c r="F2" s="215"/>
+      <c r="G2" s="215"/>
+      <c r="H2" s="215"/>
+      <c r="I2" s="216"/>
     </row>
     <row r="3" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="201"/>
-      <c r="B3" s="258"/>
-      <c r="C3" s="258"/>
-      <c r="D3" s="258"/>
-      <c r="E3" s="258"/>
-      <c r="F3" s="258"/>
-      <c r="G3" s="258"/>
-      <c r="H3" s="258"/>
+      <c r="B3" s="253"/>
+      <c r="C3" s="253"/>
+      <c r="D3" s="253"/>
+      <c r="E3" s="253"/>
+      <c r="F3" s="253"/>
+      <c r="G3" s="253"/>
+      <c r="H3" s="253"/>
       <c r="I3" s="202"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="206"/>
-      <c r="B4" s="259"/>
-      <c r="C4" s="259"/>
-      <c r="D4" s="259"/>
-      <c r="E4" s="259"/>
-      <c r="F4" s="259"/>
-      <c r="G4" s="259"/>
-      <c r="H4" s="259"/>
-      <c r="I4" s="207"/>
+      <c r="A4" s="212"/>
+      <c r="B4" s="251"/>
+      <c r="C4" s="251"/>
+      <c r="D4" s="251"/>
+      <c r="E4" s="251"/>
+      <c r="F4" s="251"/>
+      <c r="G4" s="251"/>
+      <c r="H4" s="251"/>
+      <c r="I4" s="213"/>
     </row>
     <row r="5" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="206"/>
-      <c r="B5" s="259"/>
-      <c r="C5" s="259"/>
-      <c r="D5" s="259"/>
-      <c r="E5" s="259"/>
-      <c r="F5" s="259"/>
-      <c r="G5" s="259"/>
-      <c r="H5" s="259"/>
-      <c r="I5" s="207"/>
+      <c r="A5" s="212"/>
+      <c r="B5" s="251"/>
+      <c r="C5" s="251"/>
+      <c r="D5" s="251"/>
+      <c r="E5" s="251"/>
+      <c r="F5" s="251"/>
+      <c r="G5" s="251"/>
+      <c r="H5" s="251"/>
+      <c r="I5" s="213"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="206"/>
-      <c r="B6" s="259"/>
-      <c r="C6" s="259"/>
-      <c r="D6" s="259"/>
-      <c r="E6" s="259"/>
-      <c r="F6" s="259"/>
-      <c r="G6" s="259"/>
-      <c r="H6" s="259"/>
-      <c r="I6" s="207"/>
-    </row>
-    <row r="7" spans="1:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="219"/>
-      <c r="B7" s="220"/>
-      <c r="C7" s="220"/>
-      <c r="D7" s="220"/>
-      <c r="E7" s="220"/>
-      <c r="F7" s="220"/>
-      <c r="G7" s="220"/>
-      <c r="H7" s="220"/>
-      <c r="I7" s="221"/>
+      <c r="A6" s="212"/>
+      <c r="B6" s="251"/>
+      <c r="C6" s="251"/>
+      <c r="D6" s="251"/>
+      <c r="E6" s="251"/>
+      <c r="F6" s="251"/>
+      <c r="G6" s="251"/>
+      <c r="H6" s="251"/>
+      <c r="I6" s="213"/>
+    </row>
+    <row r="7" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="212"/>
+      <c r="B7" s="251"/>
+      <c r="C7" s="251"/>
+      <c r="D7" s="251"/>
+      <c r="E7" s="251"/>
+      <c r="F7" s="251"/>
+      <c r="G7" s="251"/>
+      <c r="H7" s="251"/>
+      <c r="I7" s="213"/>
     </row>
     <row r="8" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="60" t="s">
-        <v>62</v>
-      </c>
-      <c r="B8" s="56"/>
-      <c r="C8" s="56"/>
-      <c r="D8" s="56"/>
-      <c r="E8" s="56"/>
-      <c r="F8" s="56"/>
-      <c r="G8" s="56"/>
-      <c r="H8" s="56"/>
-      <c r="I8" s="57"/>
-      <c r="K8" s="74"/>
+      <c r="A8" s="254" t="s">
+        <v>86</v>
+      </c>
+      <c r="B8" s="252"/>
+      <c r="C8" s="252"/>
+      <c r="D8" s="252"/>
+      <c r="E8" s="252"/>
+      <c r="F8" s="252"/>
+      <c r="G8" s="252"/>
+      <c r="H8" s="252"/>
+      <c r="I8" s="255"/>
+      <c r="K8" s="72"/>
     </row>
     <row r="9" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="211" t="s">
-        <v>82</v>
-      </c>
-      <c r="B9" s="260"/>
-      <c r="C9" s="260"/>
-      <c r="D9" s="260"/>
-      <c r="E9" s="260"/>
-      <c r="F9" s="260"/>
-      <c r="G9" s="260"/>
-      <c r="H9" s="260"/>
-      <c r="I9" s="213"/>
+      <c r="A9" s="203" t="s">
+        <v>90</v>
+      </c>
+      <c r="B9" s="250"/>
+      <c r="C9" s="250"/>
+      <c r="D9" s="250"/>
+      <c r="E9" s="250"/>
+      <c r="F9" s="250"/>
+      <c r="G9" s="250"/>
+      <c r="H9" s="250"/>
+      <c r="I9" s="205"/>
     </row>
     <row r="10" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="211"/>
-      <c r="B10" s="260"/>
-      <c r="C10" s="260"/>
-      <c r="D10" s="260"/>
-      <c r="E10" s="260"/>
-      <c r="F10" s="260"/>
-      <c r="G10" s="260"/>
-      <c r="H10" s="260"/>
-      <c r="I10" s="213"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" s="203"/>
+      <c r="B10" s="250"/>
+      <c r="C10" s="250"/>
+      <c r="D10" s="250"/>
+      <c r="E10" s="250"/>
+      <c r="F10" s="250"/>
+      <c r="G10" s="250"/>
+      <c r="H10" s="250"/>
+      <c r="I10" s="205"/>
+    </row>
+    <row r="11" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="198"/>
       <c r="B11" s="199"/>
       <c r="C11" s="199"/>
@@ -3669,119 +3660,119 @@
       <c r="I11" s="200"/>
     </row>
     <row r="12" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="61" t="s">
-        <v>81</v>
-      </c>
-      <c r="B12" s="261"/>
-      <c r="C12" s="261"/>
-      <c r="D12" s="261"/>
-      <c r="E12" s="261"/>
-      <c r="F12" s="261"/>
-      <c r="G12" s="261"/>
-      <c r="H12" s="261"/>
-      <c r="I12" s="73"/>
+      <c r="A12" s="254" t="s">
+        <v>82</v>
+      </c>
+      <c r="B12" s="252"/>
+      <c r="C12" s="252"/>
+      <c r="D12" s="252"/>
+      <c r="E12" s="252"/>
+      <c r="F12" s="252"/>
+      <c r="G12" s="252"/>
+      <c r="H12" s="252"/>
+      <c r="I12" s="255"/>
     </row>
     <row r="13" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="198" t="s">
-        <v>80</v>
-      </c>
-      <c r="B13" s="199"/>
-      <c r="C13" s="199"/>
-      <c r="D13" s="199"/>
-      <c r="E13" s="199"/>
-      <c r="F13" s="199"/>
-      <c r="G13" s="199"/>
-      <c r="H13" s="199"/>
-      <c r="I13" s="200"/>
-      <c r="J13" s="74"/>
+      <c r="A13" s="203" t="s">
+        <v>85</v>
+      </c>
+      <c r="B13" s="250"/>
+      <c r="C13" s="250"/>
+      <c r="D13" s="250"/>
+      <c r="E13" s="250"/>
+      <c r="F13" s="250"/>
+      <c r="G13" s="250"/>
+      <c r="H13" s="250"/>
+      <c r="I13" s="205"/>
+      <c r="J13" s="72"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="217" t="s">
+      <c r="A14" s="198"/>
+      <c r="B14" s="199"/>
+      <c r="C14" s="199"/>
+      <c r="D14" s="199"/>
+      <c r="E14" s="199"/>
+      <c r="F14" s="199"/>
+      <c r="G14" s="199"/>
+      <c r="H14" s="199"/>
+      <c r="I14" s="200"/>
+    </row>
+    <row r="15" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="196" t="s">
         <v>47</v>
       </c>
-      <c r="B14" s="256"/>
-      <c r="C14" s="256"/>
-      <c r="D14" s="256"/>
-      <c r="E14" s="256"/>
-      <c r="F14" s="256"/>
-      <c r="G14" s="256"/>
-      <c r="H14" s="256"/>
-      <c r="I14" s="218"/>
-    </row>
-    <row r="15" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="211" t="s">
-        <v>79</v>
-      </c>
-      <c r="B15" s="260"/>
-      <c r="C15" s="260"/>
-      <c r="D15" s="260"/>
-      <c r="E15" s="260"/>
-      <c r="F15" s="260"/>
-      <c r="G15" s="260"/>
-      <c r="H15" s="260"/>
-      <c r="I15" s="213"/>
+      <c r="B15" s="256"/>
+      <c r="C15" s="256"/>
+      <c r="D15" s="256"/>
+      <c r="E15" s="256"/>
+      <c r="F15" s="256"/>
+      <c r="G15" s="256"/>
+      <c r="H15" s="256"/>
+      <c r="I15" s="197"/>
     </row>
     <row r="16" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="211"/>
-      <c r="B16" s="260"/>
-      <c r="C16" s="260"/>
-      <c r="D16" s="260"/>
-      <c r="E16" s="260"/>
-      <c r="F16" s="260"/>
-      <c r="G16" s="260"/>
-      <c r="H16" s="260"/>
-      <c r="I16" s="213"/>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="211"/>
-      <c r="B17" s="260"/>
-      <c r="C17" s="260"/>
-      <c r="D17" s="260"/>
-      <c r="E17" s="260"/>
-      <c r="F17" s="260"/>
-      <c r="G17" s="260"/>
-      <c r="H17" s="260"/>
-      <c r="I17" s="213"/>
+      <c r="A16" s="203" t="s">
+        <v>74</v>
+      </c>
+      <c r="B16" s="250"/>
+      <c r="C16" s="250"/>
+      <c r="D16" s="250"/>
+      <c r="E16" s="250"/>
+      <c r="F16" s="250"/>
+      <c r="G16" s="250"/>
+      <c r="H16" s="250"/>
+      <c r="I16" s="205"/>
+    </row>
+    <row r="17" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="203"/>
+      <c r="B17" s="250"/>
+      <c r="C17" s="250"/>
+      <c r="D17" s="250"/>
+      <c r="E17" s="250"/>
+      <c r="F17" s="250"/>
+      <c r="G17" s="250"/>
+      <c r="H17" s="250"/>
+      <c r="I17" s="205"/>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="211"/>
-      <c r="B18" s="260"/>
-      <c r="C18" s="260"/>
-      <c r="D18" s="260"/>
-      <c r="E18" s="260"/>
-      <c r="F18" s="260"/>
-      <c r="G18" s="260"/>
-      <c r="H18" s="260"/>
-      <c r="I18" s="213"/>
+      <c r="A18" s="203"/>
+      <c r="B18" s="250"/>
+      <c r="C18" s="250"/>
+      <c r="D18" s="250"/>
+      <c r="E18" s="250"/>
+      <c r="F18" s="250"/>
+      <c r="G18" s="250"/>
+      <c r="H18" s="250"/>
+      <c r="I18" s="205"/>
     </row>
     <row r="19" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="214" t="s">
-        <v>67</v>
-      </c>
-      <c r="B19" s="215"/>
-      <c r="C19" s="215"/>
-      <c r="D19" s="215"/>
-      <c r="E19" s="215"/>
-      <c r="F19" s="215"/>
-      <c r="G19" s="215"/>
-      <c r="H19" s="215"/>
-      <c r="I19" s="216"/>
+      <c r="A19" s="203"/>
+      <c r="B19" s="250"/>
+      <c r="C19" s="250"/>
+      <c r="D19" s="250"/>
+      <c r="E19" s="250"/>
+      <c r="F19" s="250"/>
+      <c r="G19" s="250"/>
+      <c r="H19" s="250"/>
+      <c r="I19" s="205"/>
     </row>
     <row r="20" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="225" t="s">
-        <v>68</v>
-      </c>
-      <c r="B20" s="257"/>
-      <c r="C20" s="257"/>
-      <c r="D20" s="257"/>
-      <c r="E20" s="257"/>
-      <c r="F20" s="257"/>
-      <c r="G20" s="257"/>
-      <c r="H20" s="257"/>
-      <c r="I20" s="226"/>
+      <c r="A20" s="206" t="s">
+        <v>87</v>
+      </c>
+      <c r="B20" s="207"/>
+      <c r="C20" s="207"/>
+      <c r="D20" s="207"/>
+      <c r="E20" s="207"/>
+      <c r="F20" s="207"/>
+      <c r="G20" s="207"/>
+      <c r="H20" s="207"/>
+      <c r="I20" s="208"/>
     </row>
     <row r="21" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="225"/>
+      <c r="A21" s="220" t="s">
+        <v>84</v>
+      </c>
       <c r="B21" s="257"/>
       <c r="C21" s="257"/>
       <c r="D21" s="257"/>
@@ -3789,289 +3780,290 @@
       <c r="F21" s="257"/>
       <c r="G21" s="257"/>
       <c r="H21" s="257"/>
-      <c r="I21" s="226"/>
+      <c r="I21" s="221"/>
     </row>
     <row r="22" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="217"/>
-      <c r="B22" s="256"/>
-      <c r="C22" s="256"/>
-      <c r="D22" s="256"/>
-      <c r="E22" s="256"/>
-      <c r="F22" s="256"/>
-      <c r="G22" s="256"/>
-      <c r="H22" s="256"/>
-      <c r="I22" s="218"/>
+      <c r="A22" s="220"/>
+      <c r="B22" s="257"/>
+      <c r="C22" s="257"/>
+      <c r="D22" s="257"/>
+      <c r="E22" s="257"/>
+      <c r="F22" s="257"/>
+      <c r="G22" s="257"/>
+      <c r="H22" s="257"/>
+      <c r="I22" s="221"/>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="227"/>
-      <c r="B23" s="262"/>
-      <c r="C23" s="262"/>
-      <c r="D23" s="262"/>
-      <c r="E23" s="262"/>
-      <c r="F23" s="262"/>
-      <c r="G23" s="262"/>
-      <c r="H23" s="262"/>
-      <c r="I23" s="228"/>
+      <c r="A23" s="222"/>
+      <c r="B23" s="258"/>
+      <c r="C23" s="258"/>
+      <c r="D23" s="258"/>
+      <c r="E23" s="258"/>
+      <c r="F23" s="258"/>
+      <c r="G23" s="258"/>
+      <c r="H23" s="258"/>
+      <c r="I23" s="223"/>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="227"/>
-      <c r="B24" s="262"/>
-      <c r="C24" s="262"/>
-      <c r="D24" s="262"/>
-      <c r="E24" s="262"/>
-      <c r="F24" s="262"/>
-      <c r="G24" s="262"/>
-      <c r="H24" s="262"/>
-      <c r="I24" s="228"/>
+      <c r="A24" s="222"/>
+      <c r="B24" s="258"/>
+      <c r="C24" s="258"/>
+      <c r="D24" s="258"/>
+      <c r="E24" s="258"/>
+      <c r="F24" s="258"/>
+      <c r="G24" s="258"/>
+      <c r="H24" s="258"/>
+      <c r="I24" s="223"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="227"/>
-      <c r="B25" s="262"/>
-      <c r="C25" s="262"/>
-      <c r="D25" s="262"/>
-      <c r="E25" s="262"/>
-      <c r="F25" s="262"/>
-      <c r="G25" s="262"/>
-      <c r="H25" s="262"/>
-      <c r="I25" s="228"/>
+      <c r="A25" s="222"/>
+      <c r="B25" s="258"/>
+      <c r="C25" s="258"/>
+      <c r="D25" s="258"/>
+      <c r="E25" s="258"/>
+      <c r="F25" s="258"/>
+      <c r="G25" s="258"/>
+      <c r="H25" s="258"/>
+      <c r="I25" s="223"/>
     </row>
     <row r="26" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="201"/>
-      <c r="B26" s="258"/>
-      <c r="C26" s="258"/>
-      <c r="D26" s="258"/>
-      <c r="E26" s="258"/>
-      <c r="F26" s="258"/>
-      <c r="G26" s="258"/>
-      <c r="H26" s="258"/>
+      <c r="B26" s="253"/>
+      <c r="C26" s="253"/>
+      <c r="D26" s="253"/>
+      <c r="E26" s="253"/>
+      <c r="F26" s="253"/>
+      <c r="G26" s="253"/>
+      <c r="H26" s="253"/>
       <c r="I26" s="202"/>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="201"/>
-      <c r="B27" s="258"/>
-      <c r="C27" s="258"/>
-      <c r="D27" s="258"/>
-      <c r="E27" s="258"/>
-      <c r="F27" s="258"/>
-      <c r="G27" s="258"/>
-      <c r="H27" s="258"/>
+      <c r="B27" s="253"/>
+      <c r="C27" s="253"/>
+      <c r="D27" s="253"/>
+      <c r="E27" s="253"/>
+      <c r="F27" s="253"/>
+      <c r="G27" s="253"/>
+      <c r="H27" s="253"/>
       <c r="I27" s="202"/>
     </row>
     <row r="28" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="201"/>
-      <c r="B28" s="258"/>
-      <c r="C28" s="258"/>
-      <c r="D28" s="258"/>
-      <c r="E28" s="258"/>
-      <c r="F28" s="258"/>
-      <c r="G28" s="258"/>
-      <c r="H28" s="258"/>
+      <c r="B28" s="253"/>
+      <c r="C28" s="253"/>
+      <c r="D28" s="253"/>
+      <c r="E28" s="253"/>
+      <c r="F28" s="253"/>
+      <c r="G28" s="253"/>
+      <c r="H28" s="253"/>
       <c r="I28" s="202"/>
     </row>
     <row r="29" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="201"/>
-      <c r="B29" s="258"/>
-      <c r="C29" s="258"/>
-      <c r="D29" s="258"/>
-      <c r="E29" s="258"/>
-      <c r="F29" s="258"/>
-      <c r="G29" s="258"/>
-      <c r="H29" s="258"/>
+      <c r="B29" s="253"/>
+      <c r="C29" s="253"/>
+      <c r="D29" s="253"/>
+      <c r="E29" s="253"/>
+      <c r="F29" s="253"/>
+      <c r="G29" s="253"/>
+      <c r="H29" s="253"/>
       <c r="I29" s="202"/>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="201"/>
-      <c r="B30" s="258"/>
-      <c r="C30" s="258"/>
-      <c r="D30" s="258"/>
-      <c r="E30" s="258"/>
-      <c r="F30" s="258"/>
-      <c r="G30" s="258"/>
-      <c r="H30" s="258"/>
+      <c r="B30" s="253"/>
+      <c r="C30" s="253"/>
+      <c r="D30" s="253"/>
+      <c r="E30" s="253"/>
+      <c r="F30" s="253"/>
+      <c r="G30" s="253"/>
+      <c r="H30" s="253"/>
       <c r="I30" s="202"/>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="201"/>
-      <c r="B31" s="258"/>
-      <c r="C31" s="258"/>
-      <c r="D31" s="258"/>
-      <c r="E31" s="258"/>
-      <c r="F31" s="258"/>
-      <c r="G31" s="258"/>
-      <c r="H31" s="258"/>
+      <c r="B31" s="253"/>
+      <c r="C31" s="253"/>
+      <c r="D31" s="253"/>
+      <c r="E31" s="253"/>
+      <c r="F31" s="253"/>
+      <c r="G31" s="253"/>
+      <c r="H31" s="253"/>
       <c r="I31" s="202"/>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="201"/>
-      <c r="B32" s="258"/>
-      <c r="C32" s="258"/>
-      <c r="D32" s="258"/>
-      <c r="E32" s="258"/>
-      <c r="F32" s="258"/>
-      <c r="G32" s="258"/>
-      <c r="H32" s="258"/>
+      <c r="B32" s="253"/>
+      <c r="C32" s="253"/>
+      <c r="D32" s="253"/>
+      <c r="E32" s="253"/>
+      <c r="F32" s="253"/>
+      <c r="G32" s="253"/>
+      <c r="H32" s="253"/>
       <c r="I32" s="202"/>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="201"/>
-      <c r="B33" s="258"/>
-      <c r="C33" s="258"/>
-      <c r="D33" s="258"/>
-      <c r="E33" s="258"/>
-      <c r="F33" s="258"/>
-      <c r="G33" s="258"/>
-      <c r="H33" s="258"/>
+      <c r="B33" s="253"/>
+      <c r="C33" s="253"/>
+      <c r="D33" s="253"/>
+      <c r="E33" s="253"/>
+      <c r="F33" s="253"/>
+      <c r="G33" s="253"/>
+      <c r="H33" s="253"/>
       <c r="I33" s="202"/>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="201"/>
-      <c r="B34" s="258"/>
-      <c r="C34" s="258"/>
-      <c r="D34" s="258"/>
-      <c r="E34" s="258"/>
-      <c r="F34" s="258"/>
-      <c r="G34" s="258"/>
-      <c r="H34" s="258"/>
+      <c r="B34" s="253"/>
+      <c r="C34" s="253"/>
+      <c r="D34" s="253"/>
+      <c r="E34" s="253"/>
+      <c r="F34" s="253"/>
+      <c r="G34" s="253"/>
+      <c r="H34" s="253"/>
       <c r="I34" s="202"/>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="201"/>
-      <c r="B35" s="258"/>
-      <c r="C35" s="258"/>
-      <c r="D35" s="258"/>
-      <c r="E35" s="258"/>
-      <c r="F35" s="258"/>
-      <c r="G35" s="258"/>
-      <c r="H35" s="258"/>
+      <c r="B35" s="253"/>
+      <c r="C35" s="253"/>
+      <c r="D35" s="253"/>
+      <c r="E35" s="253"/>
+      <c r="F35" s="253"/>
+      <c r="G35" s="253"/>
+      <c r="H35" s="253"/>
       <c r="I35" s="202"/>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="201"/>
-      <c r="B36" s="258"/>
-      <c r="C36" s="258"/>
-      <c r="D36" s="258"/>
-      <c r="E36" s="258"/>
-      <c r="F36" s="258"/>
-      <c r="G36" s="258"/>
-      <c r="H36" s="258"/>
+      <c r="B36" s="253"/>
+      <c r="C36" s="253"/>
+      <c r="D36" s="253"/>
+      <c r="E36" s="253"/>
+      <c r="F36" s="253"/>
+      <c r="G36" s="253"/>
+      <c r="H36" s="253"/>
       <c r="I36" s="202"/>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="201"/>
-      <c r="B37" s="258"/>
-      <c r="C37" s="258"/>
-      <c r="D37" s="258"/>
-      <c r="E37" s="258"/>
-      <c r="F37" s="258"/>
-      <c r="G37" s="258"/>
-      <c r="H37" s="258"/>
+      <c r="B37" s="253"/>
+      <c r="C37" s="253"/>
+      <c r="D37" s="253"/>
+      <c r="E37" s="253"/>
+      <c r="F37" s="253"/>
+      <c r="G37" s="253"/>
+      <c r="H37" s="253"/>
       <c r="I37" s="202"/>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="201"/>
-      <c r="B38" s="258"/>
-      <c r="C38" s="258"/>
-      <c r="D38" s="258"/>
-      <c r="E38" s="258"/>
-      <c r="F38" s="258"/>
-      <c r="G38" s="258"/>
-      <c r="H38" s="258"/>
+      <c r="B38" s="253"/>
+      <c r="C38" s="253"/>
+      <c r="D38" s="253"/>
+      <c r="E38" s="253"/>
+      <c r="F38" s="253"/>
+      <c r="G38" s="253"/>
+      <c r="H38" s="253"/>
       <c r="I38" s="202"/>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="201"/>
-      <c r="B39" s="258"/>
-      <c r="C39" s="258"/>
-      <c r="D39" s="258"/>
-      <c r="E39" s="258"/>
-      <c r="F39" s="258"/>
-      <c r="G39" s="258"/>
-      <c r="H39" s="258"/>
+      <c r="B39" s="253"/>
+      <c r="C39" s="253"/>
+      <c r="D39" s="253"/>
+      <c r="E39" s="253"/>
+      <c r="F39" s="253"/>
+      <c r="G39" s="253"/>
+      <c r="H39" s="253"/>
       <c r="I39" s="202"/>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="201"/>
-      <c r="B40" s="258"/>
-      <c r="C40" s="258"/>
-      <c r="D40" s="258"/>
-      <c r="E40" s="258"/>
-      <c r="F40" s="258"/>
-      <c r="G40" s="258"/>
-      <c r="H40" s="258"/>
+      <c r="B40" s="253"/>
+      <c r="C40" s="253"/>
+      <c r="D40" s="253"/>
+      <c r="E40" s="253"/>
+      <c r="F40" s="253"/>
+      <c r="G40" s="253"/>
+      <c r="H40" s="253"/>
       <c r="I40" s="202"/>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="201"/>
-      <c r="B41" s="258"/>
-      <c r="C41" s="258"/>
-      <c r="D41" s="258"/>
-      <c r="E41" s="258"/>
-      <c r="F41" s="258"/>
-      <c r="G41" s="258"/>
-      <c r="H41" s="258"/>
+      <c r="B41" s="253"/>
+      <c r="C41" s="253"/>
+      <c r="D41" s="253"/>
+      <c r="E41" s="253"/>
+      <c r="F41" s="253"/>
+      <c r="G41" s="253"/>
+      <c r="H41" s="253"/>
       <c r="I41" s="202"/>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="201"/>
-      <c r="B42" s="258"/>
-      <c r="C42" s="258"/>
-      <c r="D42" s="258"/>
-      <c r="E42" s="258"/>
-      <c r="F42" s="258"/>
-      <c r="G42" s="258"/>
-      <c r="H42" s="258"/>
+      <c r="B42" s="253"/>
+      <c r="C42" s="253"/>
+      <c r="D42" s="253"/>
+      <c r="E42" s="253"/>
+      <c r="F42" s="253"/>
+      <c r="G42" s="253"/>
+      <c r="H42" s="253"/>
       <c r="I42" s="202"/>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="201"/>
-      <c r="B43" s="258"/>
-      <c r="C43" s="258"/>
-      <c r="D43" s="258"/>
-      <c r="E43" s="258"/>
-      <c r="F43" s="258"/>
-      <c r="G43" s="258"/>
-      <c r="H43" s="258"/>
+      <c r="B43" s="253"/>
+      <c r="C43" s="253"/>
+      <c r="D43" s="253"/>
+      <c r="E43" s="253"/>
+      <c r="F43" s="253"/>
+      <c r="G43" s="253"/>
+      <c r="H43" s="253"/>
       <c r="I43" s="202"/>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="201"/>
-      <c r="B44" s="258"/>
-      <c r="C44" s="258"/>
-      <c r="D44" s="258"/>
-      <c r="E44" s="258"/>
-      <c r="F44" s="258"/>
-      <c r="G44" s="258"/>
-      <c r="H44" s="258"/>
+      <c r="B44" s="253"/>
+      <c r="C44" s="253"/>
+      <c r="D44" s="253"/>
+      <c r="E44" s="253"/>
+      <c r="F44" s="253"/>
+      <c r="G44" s="253"/>
+      <c r="H44" s="253"/>
       <c r="I44" s="202"/>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="201"/>
-      <c r="B45" s="258"/>
-      <c r="C45" s="258"/>
-      <c r="D45" s="258"/>
-      <c r="E45" s="258"/>
-      <c r="F45" s="258"/>
-      <c r="G45" s="258"/>
-      <c r="H45" s="258"/>
+      <c r="B45" s="253"/>
+      <c r="C45" s="253"/>
+      <c r="D45" s="253"/>
+      <c r="E45" s="253"/>
+      <c r="F45" s="253"/>
+      <c r="G45" s="253"/>
+      <c r="H45" s="253"/>
       <c r="I45" s="202"/>
     </row>
     <row r="46" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="222"/>
-      <c r="B46" s="223"/>
-      <c r="C46" s="223"/>
-      <c r="D46" s="223"/>
-      <c r="E46" s="223"/>
-      <c r="F46" s="223"/>
-      <c r="G46" s="223"/>
-      <c r="H46" s="223"/>
-      <c r="I46" s="224"/>
+      <c r="A46" s="217"/>
+      <c r="B46" s="218"/>
+      <c r="C46" s="218"/>
+      <c r="D46" s="218"/>
+      <c r="E46" s="218"/>
+      <c r="F46" s="218"/>
+      <c r="G46" s="218"/>
+      <c r="H46" s="218"/>
+      <c r="I46" s="219"/>
     </row>
   </sheetData>
-  <mergeCells count="36">
+  <mergeCells count="35">
+    <mergeCell ref="A9:I11"/>
+    <mergeCell ref="A13:I14"/>
     <mergeCell ref="A7:I7"/>
-    <mergeCell ref="A9:I11"/>
     <mergeCell ref="A46:I46"/>
-    <mergeCell ref="A20:I21"/>
+    <mergeCell ref="A21:I22"/>
     <mergeCell ref="A23:I25"/>
     <mergeCell ref="A41:I41"/>
     <mergeCell ref="A42:I42"/>
@@ -4090,7 +4082,6 @@
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="A6:I6"/>
     <mergeCell ref="A5:I5"/>
-    <mergeCell ref="A13:I13"/>
     <mergeCell ref="A35:I35"/>
     <mergeCell ref="A26:I26"/>
     <mergeCell ref="A27:I27"/>
@@ -4099,10 +4090,9 @@
     <mergeCell ref="A33:I33"/>
     <mergeCell ref="A34:I34"/>
     <mergeCell ref="A30:I30"/>
-    <mergeCell ref="A15:I18"/>
-    <mergeCell ref="A19:I19"/>
-    <mergeCell ref="A22:I22"/>
-    <mergeCell ref="A14:I14"/>
+    <mergeCell ref="A16:I19"/>
+    <mergeCell ref="A20:I20"/>
+    <mergeCell ref="A15:I15"/>
     <mergeCell ref="A32:I32"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4119,106 +4109,106 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="238" t="s">
+      <c r="A1" s="233" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="239"/>
-      <c r="C1" s="239"/>
-      <c r="D1" s="240"/>
-      <c r="E1" s="247" t="s">
-        <v>83</v>
-      </c>
-      <c r="F1" s="248"/>
+      <c r="B1" s="234"/>
+      <c r="C1" s="234"/>
+      <c r="D1" s="235"/>
+      <c r="E1" s="241" t="s">
+        <v>75</v>
+      </c>
+      <c r="F1" s="242"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="208" t="s">
+      <c r="A2" s="214" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="209"/>
-      <c r="C2" s="209"/>
-      <c r="D2" s="209"/>
-      <c r="E2" s="209"/>
-      <c r="F2" s="209"/>
-      <c r="G2" s="209"/>
-      <c r="H2" s="209"/>
-      <c r="I2" s="210"/>
+      <c r="B2" s="215"/>
+      <c r="C2" s="215"/>
+      <c r="D2" s="215"/>
+      <c r="E2" s="215"/>
+      <c r="F2" s="215"/>
+      <c r="G2" s="215"/>
+      <c r="H2" s="215"/>
+      <c r="I2" s="216"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="229" t="s">
+      <c r="A3" s="224" t="s">
         <v>49</v>
       </c>
-      <c r="B3" s="230"/>
-      <c r="C3" s="230"/>
-      <c r="D3" s="230"/>
-      <c r="E3" s="230"/>
-      <c r="F3" s="230"/>
-      <c r="G3" s="230"/>
-      <c r="H3" s="230"/>
-      <c r="I3" s="231"/>
-      <c r="K3" s="74"/>
+      <c r="B3" s="225"/>
+      <c r="C3" s="225"/>
+      <c r="D3" s="225"/>
+      <c r="E3" s="225"/>
+      <c r="F3" s="225"/>
+      <c r="G3" s="225"/>
+      <c r="H3" s="225"/>
+      <c r="I3" s="226"/>
+      <c r="K3" s="72"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="214" t="s">
+      <c r="A4" s="206" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="215"/>
-      <c r="C4" s="215"/>
-      <c r="D4" s="215"/>
-      <c r="E4" s="215"/>
-      <c r="F4" s="215"/>
-      <c r="G4" s="215"/>
-      <c r="H4" s="215"/>
-      <c r="I4" s="216"/>
+      <c r="B4" s="207"/>
+      <c r="C4" s="207"/>
+      <c r="D4" s="207"/>
+      <c r="E4" s="207"/>
+      <c r="F4" s="207"/>
+      <c r="G4" s="207"/>
+      <c r="H4" s="207"/>
+      <c r="I4" s="208"/>
     </row>
     <row r="5" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="61" t="s">
-        <v>84</v>
-      </c>
-      <c r="B5" s="62"/>
-      <c r="C5" s="62"/>
-      <c r="D5" s="62"/>
-      <c r="E5" s="62"/>
-      <c r="F5" s="62"/>
-      <c r="G5" s="62"/>
-      <c r="H5" s="62"/>
-      <c r="I5" s="63"/>
+      <c r="A5" s="60" t="s">
+        <v>76</v>
+      </c>
+      <c r="B5" s="61"/>
+      <c r="C5" s="61"/>
+      <c r="D5" s="61"/>
+      <c r="E5" s="61"/>
+      <c r="F5" s="61"/>
+      <c r="G5" s="61"/>
+      <c r="H5" s="61"/>
+      <c r="I5" s="62"/>
     </row>
     <row r="6" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="65" t="s">
-        <v>85</v>
+      <c r="A6" s="64" t="s">
+        <v>77</v>
       </c>
       <c r="B6" s="56"/>
       <c r="C6" s="56"/>
       <c r="D6" s="56"/>
-      <c r="E6" s="64"/>
+      <c r="E6" s="63"/>
       <c r="F6" s="56"/>
       <c r="G6" s="56"/>
       <c r="H6" s="56"/>
       <c r="I6" s="57"/>
     </row>
     <row r="7" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="211" t="s">
-        <v>86</v>
-      </c>
-      <c r="B7" s="212"/>
-      <c r="C7" s="212"/>
-      <c r="D7" s="212"/>
-      <c r="E7" s="212"/>
-      <c r="F7" s="212"/>
-      <c r="G7" s="212"/>
-      <c r="H7" s="212"/>
-      <c r="I7" s="213"/>
+      <c r="A7" s="203" t="s">
+        <v>83</v>
+      </c>
+      <c r="B7" s="250"/>
+      <c r="C7" s="250"/>
+      <c r="D7" s="250"/>
+      <c r="E7" s="250"/>
+      <c r="F7" s="250"/>
+      <c r="G7" s="250"/>
+      <c r="H7" s="250"/>
+      <c r="I7" s="205"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="211"/>
-      <c r="B8" s="212"/>
-      <c r="C8" s="212"/>
-      <c r="D8" s="212"/>
-      <c r="E8" s="212"/>
-      <c r="F8" s="212"/>
-      <c r="G8" s="212"/>
-      <c r="H8" s="212"/>
-      <c r="I8" s="213"/>
+      <c r="A8" s="203"/>
+      <c r="B8" s="250"/>
+      <c r="C8" s="250"/>
+      <c r="D8" s="250"/>
+      <c r="E8" s="250"/>
+      <c r="F8" s="250"/>
+      <c r="G8" s="250"/>
+      <c r="H8" s="250"/>
+      <c r="I8" s="205"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="198"/>
@@ -4232,21 +4222,21 @@
       <c r="I9" s="200"/>
     </row>
     <row r="10" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="232" t="s">
+      <c r="A10" s="227" t="s">
         <v>52</v>
       </c>
-      <c r="B10" s="233"/>
-      <c r="C10" s="233"/>
-      <c r="D10" s="233"/>
-      <c r="E10" s="233"/>
-      <c r="F10" s="233"/>
-      <c r="G10" s="233"/>
-      <c r="H10" s="233"/>
-      <c r="I10" s="234"/>
+      <c r="B10" s="228"/>
+      <c r="C10" s="228"/>
+      <c r="D10" s="228"/>
+      <c r="E10" s="228"/>
+      <c r="F10" s="228"/>
+      <c r="G10" s="228"/>
+      <c r="H10" s="228"/>
+      <c r="I10" s="229"/>
     </row>
     <row r="11" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="198" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B11" s="199"/>
       <c r="C11" s="199"/>
@@ -4258,218 +4248,217 @@
       <c r="I11" s="200"/>
     </row>
     <row r="12" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="244" t="s">
+      <c r="A12" s="239" t="s">
         <v>53</v>
       </c>
-      <c r="B12" s="245"/>
-      <c r="C12" s="245"/>
-      <c r="D12" s="245"/>
-      <c r="E12" s="245"/>
-      <c r="F12" s="245"/>
-      <c r="G12" s="245"/>
-      <c r="H12" s="245"/>
-      <c r="I12" s="246"/>
-    </row>
-    <row r="13" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="198" t="s">
-        <v>69</v>
-      </c>
-      <c r="B13" s="199"/>
-      <c r="C13" s="199"/>
-      <c r="D13" s="199"/>
-      <c r="E13" s="199"/>
-      <c r="F13" s="199"/>
-      <c r="G13" s="199"/>
-      <c r="H13" s="199"/>
-      <c r="I13" s="200"/>
+      <c r="B12" s="259"/>
+      <c r="C12" s="259"/>
+      <c r="D12" s="259"/>
+      <c r="E12" s="259"/>
+      <c r="F12" s="259"/>
+      <c r="G12" s="259"/>
+      <c r="H12" s="259"/>
+      <c r="I12" s="240"/>
+    </row>
+    <row r="13" spans="1:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="230" t="s">
+        <v>89</v>
+      </c>
+      <c r="B13" s="231"/>
+      <c r="C13" s="231"/>
+      <c r="D13" s="231"/>
+      <c r="E13" s="231"/>
+      <c r="F13" s="231"/>
+      <c r="G13" s="231"/>
+      <c r="H13" s="231"/>
+      <c r="I13" s="232"/>
     </row>
     <row r="14" spans="1:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="15" spans="1:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="241" t="s">
+      <c r="A15" s="236" t="s">
         <v>54</v>
       </c>
-      <c r="B15" s="242"/>
-      <c r="C15" s="242"/>
-      <c r="D15" s="243"/>
-      <c r="E15" s="247" t="s">
-        <v>83</v>
-      </c>
-      <c r="F15" s="248"/>
-      <c r="K15" s="74"/>
+      <c r="B15" s="237"/>
+      <c r="C15" s="237"/>
+      <c r="D15" s="238"/>
+      <c r="E15" s="241" t="s">
+        <v>75</v>
+      </c>
+      <c r="F15" s="242"/>
     </row>
     <row r="16" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="208" t="s">
+      <c r="A16" s="214" t="s">
         <v>48</v>
       </c>
-      <c r="B16" s="209"/>
-      <c r="C16" s="209"/>
-      <c r="D16" s="209"/>
-      <c r="E16" s="209"/>
-      <c r="F16" s="209"/>
-      <c r="G16" s="209"/>
-      <c r="H16" s="209"/>
-      <c r="I16" s="210"/>
+      <c r="B16" s="215"/>
+      <c r="C16" s="215"/>
+      <c r="D16" s="215"/>
+      <c r="E16" s="215"/>
+      <c r="F16" s="215"/>
+      <c r="G16" s="215"/>
+      <c r="H16" s="215"/>
+      <c r="I16" s="216"/>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="229" t="s">
-        <v>88</v>
-      </c>
-      <c r="B17" s="230"/>
-      <c r="C17" s="230"/>
-      <c r="D17" s="230"/>
-      <c r="E17" s="230"/>
-      <c r="F17" s="230"/>
-      <c r="G17" s="230"/>
-      <c r="H17" s="230"/>
-      <c r="I17" s="231"/>
+      <c r="A17" s="224" t="s">
+        <v>78</v>
+      </c>
+      <c r="B17" s="225"/>
+      <c r="C17" s="225"/>
+      <c r="D17" s="225"/>
+      <c r="E17" s="225"/>
+      <c r="F17" s="225"/>
+      <c r="G17" s="225"/>
+      <c r="H17" s="225"/>
+      <c r="I17" s="226"/>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="61" t="s">
+      <c r="A18" s="60" t="s">
         <v>39</v>
       </c>
-      <c r="B18" s="62"/>
-      <c r="C18" s="62"/>
-      <c r="D18" s="62"/>
-      <c r="E18" s="62"/>
-      <c r="F18" s="62"/>
-      <c r="G18" s="62"/>
-      <c r="H18" s="62"/>
-      <c r="I18" s="63"/>
+      <c r="B18" s="61"/>
+      <c r="C18" s="61"/>
+      <c r="D18" s="61"/>
+      <c r="E18" s="61"/>
+      <c r="F18" s="61"/>
+      <c r="G18" s="61"/>
+      <c r="H18" s="61"/>
+      <c r="I18" s="62"/>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="61" t="s">
-        <v>89</v>
-      </c>
-      <c r="B19" s="62"/>
-      <c r="C19" s="62"/>
-      <c r="D19" s="62"/>
-      <c r="E19" s="62"/>
-      <c r="F19" s="62"/>
-      <c r="G19" s="62"/>
-      <c r="H19" s="62"/>
-      <c r="I19" s="63"/>
+      <c r="A19" s="60" t="s">
+        <v>79</v>
+      </c>
+      <c r="B19" s="61"/>
+      <c r="C19" s="61"/>
+      <c r="D19" s="61"/>
+      <c r="E19" s="61"/>
+      <c r="F19" s="61"/>
+      <c r="G19" s="61"/>
+      <c r="H19" s="61"/>
+      <c r="I19" s="62"/>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="214" t="s">
+      <c r="A20" s="206" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="215"/>
-      <c r="C20" s="215"/>
-      <c r="D20" s="215"/>
-      <c r="E20" s="215"/>
-      <c r="F20" s="215"/>
-      <c r="G20" s="215"/>
-      <c r="H20" s="215"/>
-      <c r="I20" s="216"/>
+      <c r="B20" s="207"/>
+      <c r="C20" s="207"/>
+      <c r="D20" s="207"/>
+      <c r="E20" s="207"/>
+      <c r="F20" s="207"/>
+      <c r="G20" s="207"/>
+      <c r="H20" s="207"/>
+      <c r="I20" s="208"/>
     </row>
     <row r="21" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="61" t="s">
+      <c r="A21" s="60" t="s">
         <v>55</v>
       </c>
-      <c r="B21" s="62"/>
-      <c r="C21" s="62"/>
-      <c r="D21" s="62"/>
-      <c r="E21" s="62"/>
-      <c r="F21" s="62"/>
-      <c r="G21" s="62"/>
-      <c r="H21" s="62"/>
-      <c r="I21" s="63"/>
+      <c r="B21" s="61"/>
+      <c r="C21" s="61"/>
+      <c r="D21" s="61"/>
+      <c r="E21" s="61"/>
+      <c r="F21" s="61"/>
+      <c r="G21" s="61"/>
+      <c r="H21" s="61"/>
+      <c r="I21" s="62"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="65" t="s">
+      <c r="A22" s="64" t="s">
         <v>56</v>
       </c>
       <c r="B22" s="56"/>
       <c r="C22" s="56"/>
       <c r="D22" s="56"/>
-      <c r="E22" s="64"/>
+      <c r="E22" s="63"/>
       <c r="F22" s="56"/>
       <c r="G22" s="56"/>
       <c r="H22" s="56"/>
       <c r="I22" s="57"/>
     </row>
     <row r="23" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="211" t="s">
-        <v>90</v>
-      </c>
-      <c r="B23" s="212"/>
-      <c r="C23" s="212"/>
-      <c r="D23" s="212"/>
-      <c r="E23" s="212"/>
-      <c r="F23" s="212"/>
-      <c r="G23" s="212"/>
-      <c r="H23" s="212"/>
-      <c r="I23" s="213"/>
+      <c r="A23" s="203" t="s">
+        <v>80</v>
+      </c>
+      <c r="B23" s="204"/>
+      <c r="C23" s="204"/>
+      <c r="D23" s="204"/>
+      <c r="E23" s="204"/>
+      <c r="F23" s="204"/>
+      <c r="G23" s="204"/>
+      <c r="H23" s="204"/>
+      <c r="I23" s="205"/>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="211"/>
-      <c r="B24" s="212"/>
-      <c r="C24" s="212"/>
-      <c r="D24" s="212"/>
-      <c r="E24" s="212"/>
-      <c r="F24" s="212"/>
-      <c r="G24" s="212"/>
-      <c r="H24" s="212"/>
-      <c r="I24" s="213"/>
+      <c r="A24" s="203"/>
+      <c r="B24" s="204"/>
+      <c r="C24" s="204"/>
+      <c r="D24" s="204"/>
+      <c r="E24" s="204"/>
+      <c r="F24" s="204"/>
+      <c r="G24" s="204"/>
+      <c r="H24" s="204"/>
+      <c r="I24" s="205"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="211"/>
-      <c r="B25" s="212"/>
-      <c r="C25" s="212"/>
-      <c r="D25" s="212"/>
-      <c r="E25" s="212"/>
-      <c r="F25" s="212"/>
-      <c r="G25" s="212"/>
-      <c r="H25" s="212"/>
-      <c r="I25" s="213"/>
+      <c r="A25" s="203"/>
+      <c r="B25" s="204"/>
+      <c r="C25" s="204"/>
+      <c r="D25" s="204"/>
+      <c r="E25" s="204"/>
+      <c r="F25" s="204"/>
+      <c r="G25" s="204"/>
+      <c r="H25" s="204"/>
+      <c r="I25" s="205"/>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="232" t="s">
+      <c r="A26" s="227" t="s">
         <v>57</v>
       </c>
-      <c r="B26" s="233"/>
-      <c r="C26" s="233"/>
-      <c r="D26" s="233"/>
-      <c r="E26" s="233"/>
-      <c r="F26" s="233"/>
-      <c r="G26" s="233"/>
-      <c r="H26" s="233"/>
-      <c r="I26" s="234"/>
+      <c r="B26" s="228"/>
+      <c r="C26" s="228"/>
+      <c r="D26" s="228"/>
+      <c r="E26" s="228"/>
+      <c r="F26" s="228"/>
+      <c r="G26" s="228"/>
+      <c r="H26" s="228"/>
+      <c r="I26" s="229"/>
     </row>
     <row r="27" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="211" t="s">
-        <v>66</v>
-      </c>
-      <c r="B27" s="212"/>
-      <c r="C27" s="212"/>
-      <c r="D27" s="212"/>
-      <c r="E27" s="212"/>
-      <c r="F27" s="212"/>
-      <c r="G27" s="212"/>
-      <c r="H27" s="212"/>
-      <c r="I27" s="213"/>
+      <c r="A27" s="203" t="s">
+        <v>81</v>
+      </c>
+      <c r="B27" s="204"/>
+      <c r="C27" s="204"/>
+      <c r="D27" s="204"/>
+      <c r="E27" s="204"/>
+      <c r="F27" s="204"/>
+      <c r="G27" s="204"/>
+      <c r="H27" s="204"/>
+      <c r="I27" s="205"/>
     </row>
     <row r="28" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="211"/>
-      <c r="B28" s="212"/>
-      <c r="C28" s="212"/>
-      <c r="D28" s="212"/>
-      <c r="E28" s="212"/>
-      <c r="F28" s="212"/>
-      <c r="G28" s="212"/>
-      <c r="H28" s="212"/>
-      <c r="I28" s="213"/>
+      <c r="A28" s="203"/>
+      <c r="B28" s="204"/>
+      <c r="C28" s="204"/>
+      <c r="D28" s="204"/>
+      <c r="E28" s="204"/>
+      <c r="F28" s="204"/>
+      <c r="G28" s="204"/>
+      <c r="H28" s="204"/>
+      <c r="I28" s="205"/>
     </row>
     <row r="29" spans="1:9" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="235"/>
-      <c r="B29" s="236"/>
-      <c r="C29" s="236"/>
-      <c r="D29" s="236"/>
-      <c r="E29" s="236"/>
-      <c r="F29" s="236"/>
-      <c r="G29" s="236"/>
-      <c r="H29" s="236"/>
-      <c r="I29" s="237"/>
+      <c r="A29" s="230"/>
+      <c r="B29" s="231"/>
+      <c r="C29" s="231"/>
+      <c r="D29" s="231"/>
+      <c r="E29" s="231"/>
+      <c r="F29" s="231"/>
+      <c r="G29" s="231"/>
+      <c r="H29" s="231"/>
+      <c r="I29" s="232"/>
     </row>
   </sheetData>
   <mergeCells count="18">
@@ -4520,18 +4509,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="250" t="s">
+      <c r="A1" s="244" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="251"/>
-      <c r="C1" s="252"/>
-      <c r="E1" s="250" t="s">
+      <c r="B1" s="245"/>
+      <c r="C1" s="246"/>
+      <c r="E1" s="244" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="251"/>
-      <c r="G1" s="252"/>
-      <c r="H1" s="249"/>
-      <c r="I1" s="249"/>
+      <c r="F1" s="245"/>
+      <c r="G1" s="246"/>
+      <c r="H1" s="243"/>
+      <c r="I1" s="243"/>
       <c r="J1" s="1"/>
     </row>
     <row r="2" spans="1:15" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4572,10 +4561,10 @@
       <c r="G3" s="12">
         <v>0</v>
       </c>
-      <c r="N3" s="254" t="s">
+      <c r="N3" s="248" t="s">
         <v>10</v>
       </c>
-      <c r="O3" s="252" t="s">
+      <c r="O3" s="246" t="s">
         <v>15</v>
       </c>
     </row>
@@ -4599,8 +4588,8 @@
         <v>0</v>
       </c>
       <c r="M4" s="27"/>
-      <c r="N4" s="255"/>
-      <c r="O4" s="253"/>
+      <c r="N4" s="249"/>
+      <c r="O4" s="247"/>
     </row>
     <row r="5" spans="1:15" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">

</xml_diff>